<commit_message>
data.xlsx has Pivot Table
</commit_message>
<xml_diff>
--- a/Excel/data.xlsx
+++ b/Excel/data.xlsx
@@ -1,21 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chimm\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chimm\Documents\DataAnalytics-2026\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{455DB51B-CFA1-4BB1-9EF7-6ABC6099A74F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{02AEB3D3-0E50-4E99-9077-19D458BAB963}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{F941E7D7-CFC5-44F0-AFA2-7AEBCB9EF5D2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="2" xr2:uid="{F941E7D7-CFC5-44F0-AFA2-7AEBCB9EF5D2}"/>
   </bookViews>
   <sheets>
-    <sheet name="raw-data" sheetId="1" r:id="rId1"/>
+    <sheet name="dataset-1" sheetId="1" r:id="rId1"/>
+    <sheet name="dataset-2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
+  <pivotCaches>
+    <pivotCache cacheId="0" r:id="rId4"/>
+  </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,32 +41,59 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="29">
   <si>
     <t>Dataset</t>
   </si>
   <si>
+    <t>Descript Stats</t>
+  </si>
+  <si>
     <t>Student</t>
   </si>
   <si>
+    <t>Score</t>
+  </si>
+  <si>
+    <t>Maximum</t>
+  </si>
+  <si>
     <t>Student 1</t>
   </si>
   <si>
+    <t>Minimum</t>
+  </si>
+  <si>
     <t>Student 2</t>
   </si>
   <si>
+    <t>Range</t>
+  </si>
+  <si>
     <t>Student 3</t>
   </si>
   <si>
+    <t>Average</t>
+  </si>
+  <si>
     <t>Student 4</t>
   </si>
   <si>
+    <t>Median</t>
+  </si>
+  <si>
     <t>Student 5</t>
   </si>
   <si>
+    <t>Mode</t>
+  </si>
+  <si>
     <t>Student 6</t>
   </si>
   <si>
+    <t>Standard Dev</t>
+  </si>
+  <si>
     <t>Student 7</t>
   </si>
   <si>
@@ -74,31 +106,28 @@
     <t>Student 10</t>
   </si>
   <si>
-    <t>Score</t>
-  </si>
-  <si>
-    <t>Descript Stats</t>
-  </si>
-  <si>
-    <t>Maximum</t>
-  </si>
-  <si>
-    <t>Minimum</t>
-  </si>
-  <si>
-    <t>Range</t>
-  </si>
-  <si>
-    <t>Average</t>
-  </si>
-  <si>
-    <t>Median</t>
-  </si>
-  <si>
-    <t>Mode</t>
-  </si>
-  <si>
-    <t>Standard Dev</t>
+    <t>Track</t>
+  </si>
+  <si>
+    <t>Time Zone</t>
+  </si>
+  <si>
+    <t>AppDev</t>
+  </si>
+  <si>
+    <t>EST</t>
+  </si>
+  <si>
+    <t>CST</t>
+  </si>
+  <si>
+    <t>Data Analytics</t>
+  </si>
+  <si>
+    <t>PST</t>
+  </si>
+  <si>
+    <t>Average of Score</t>
   </si>
 </sst>
 </file>
@@ -140,9 +169,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -158,6 +188,188 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Excel Services" refreshedDate="46108.494335069445" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="10" xr:uid="{50495AE7-B8A2-4ECD-9119-1E084F34A78A}">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A1:D11" sheet="dataset-2"/>
+  </cacheSource>
+  <cacheFields count="4">
+    <cacheField name="Student" numFmtId="0">
+      <sharedItems count="10">
+        <s v="Student 1"/>
+        <s v="Student 2"/>
+        <s v="Student 3"/>
+        <s v="Student 4"/>
+        <s v="Student 5"/>
+        <s v="Student 6"/>
+        <s v="Student 7"/>
+        <s v="Student 8"/>
+        <s v="Student 9"/>
+        <s v="Student 10"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Score" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="65" maxValue="95"/>
+    </cacheField>
+    <cacheField name="Track" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+    <cacheField name="Time Zone" numFmtId="0">
+      <sharedItems/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="10">
+  <r>
+    <x v="0"/>
+    <n v="65"/>
+    <s v="AppDev"/>
+    <s v="EST"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <n v="70"/>
+    <s v="AppDev"/>
+    <s v="CST"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <n v="75"/>
+    <s v="Data Analytics"/>
+    <s v="PST"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <n v="80"/>
+    <s v="Data Analytics"/>
+    <s v="EST"/>
+  </r>
+  <r>
+    <x v="4"/>
+    <n v="85"/>
+    <s v="AppDev"/>
+    <s v="EST"/>
+  </r>
+  <r>
+    <x v="5"/>
+    <n v="90"/>
+    <s v="AppDev"/>
+    <s v="PST"/>
+  </r>
+  <r>
+    <x v="6"/>
+    <n v="75"/>
+    <s v="AppDev"/>
+    <s v="EST"/>
+  </r>
+  <r>
+    <x v="7"/>
+    <n v="80"/>
+    <s v="Data Analytics"/>
+    <s v="PST"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <n v="95"/>
+    <s v="Data Analytics"/>
+    <s v="EST"/>
+  </r>
+  <r>
+    <x v="9"/>
+    <n v="70"/>
+    <s v="AppDev"/>
+    <s v="CST"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{63C01CC5-56EC-47D9-A33A-BA5328E30AD4}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" grandTotalCaption="Average" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+  <location ref="A2:B13" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="4">
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0">
+      <items count="11">
+        <item x="0"/>
+        <item x="9"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="11">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Average of Score" fld="1" subtotal="average" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -491,18 +703,18 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>13</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="D2">
         <f>MAX(B3:B12)</f>
@@ -511,13 +723,13 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B3">
         <v>65</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="D3">
         <f>MIN(B3:B12)</f>
@@ -526,13 +738,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B4">
         <v>70</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="D4">
         <f>D2-D3</f>
@@ -541,13 +753,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B5">
         <v>75</v>
       </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="D5">
         <f>AVERAGE(B3:B12)</f>
@@ -556,13 +768,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B6">
         <v>80</v>
       </c>
       <c r="C6" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="D6">
         <f>MEDIAN(B3:B12)</f>
@@ -571,13 +783,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="B7">
         <v>85</v>
       </c>
       <c r="C7" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="D7">
         <f>_xlfn.MODE.SNGL(B3:B12)</f>
@@ -586,13 +798,13 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="B8">
         <v>90</v>
       </c>
       <c r="C8" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D8" s="1">
         <f>_xlfn.STDEV.P(B3:B12)</f>
@@ -601,7 +813,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="B9">
         <v>75</v>
@@ -609,7 +821,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="B10">
         <v>80</v>
@@ -617,7 +829,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="B11">
         <v>95</v>
@@ -625,7 +837,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="B12">
         <v>70</v>
@@ -635,4 +847,283 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33028230-7FF2-4B04-B07B-A157F3AD123B}">
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2">
+        <v>65</v>
+      </c>
+      <c r="C2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3">
+        <v>70</v>
+      </c>
+      <c r="C3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
+        <v>75</v>
+      </c>
+      <c r="C4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5">
+        <v>80</v>
+      </c>
+      <c r="C5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6">
+        <v>85</v>
+      </c>
+      <c r="C6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7">
+        <v>90</v>
+      </c>
+      <c r="C7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8">
+        <v>75</v>
+      </c>
+      <c r="C8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9">
+        <v>80</v>
+      </c>
+      <c r="C9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D9" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10">
+        <v>95</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11">
+        <v>70</v>
+      </c>
+      <c r="C11" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{718F05EE-2EE1-410A-B16A-B3622E5053C3}">
+  <dimension ref="A2:B13"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13">
+        <v>78.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>